<commit_message>
fix error and make more accurate
</commit_message>
<xml_diff>
--- a/uploads/Chile/result-Chile FMC Vairav-OMP.xlsx.xlsx
+++ b/uploads/Chile/result-Chile FMC Vairav-OMP.xlsx.xlsx
@@ -1407,7 +1407,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1429,13 +1429,6 @@
       <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1870,19 +1863,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1891,7 +1884,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1900,125 +1896,122 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2405,8 +2398,8 @@
   <dimension ref="A1:E225"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="1" max="1" width="67.8181818181818" customWidth="1"/>
+    <col min="2" max="2" width="29.0909090909091" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
@@ -5915,7 +5908,7 @@
       </c>
     </row>
     <row r="207" spans="1:5">
-      <c r="A207" s="1" t="s">
+      <c r="A207" s="2" t="s">
         <v>418</v>
       </c>
       <c r="B207" t="s">
@@ -5925,7 +5918,7 @@
         <v>200</v>
       </c>
       <c r="D207" t="s">
-        <v>238</v>
+        <v>7</v>
       </c>
       <c r="E207" t="s">
         <v>419</v>

</xml_diff>